<commit_message>
feat: update AAA and SNMP group names to TACACS_SERVERS and SNMPv3 groups
</commit_message>
<xml_diff>
--- a/assets/sample_intent.xlsx
+++ b/assets/sample_intent.xlsx
@@ -1035,7 +1035,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>AAA_NOC</t>
+          <t>TACACS_SERVERS</t>
         </is>
       </c>
     </row>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>ROGROUP</t>
+          <t>SNMPv3_RO</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>RONMS</t>
+          <t>snmp-ro-user</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>RWGROUP</t>
+          <t>SNMPv3_RW</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1179,7 @@
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>RWNMS</t>
+          <t>snmp-rw-user</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>noc@demo.nautomation.local</t>
+          <t>netops@demo.nautomation.local</t>
         </is>
       </c>
     </row>
@@ -2902,7 +2902,7 @@
       </c>
       <c r="B2" s="12" t="inlineStr">
         <is>
-          <t>NOC management range</t>
+          <t>Management hosts</t>
         </is>
       </c>
       <c r="C2" s="12" t="inlineStr">

</xml_diff>

<commit_message>
feat: add new features for AAA, SNMP, NTP, DHCP snooping, spanning tree, and banner configurations
</commit_message>
<xml_diff>
--- a/assets/sample_intent.xlsx
+++ b/assets/sample_intent.xlsx
@@ -688,7 +688,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Toggle which config sections to generate (Yes/No). Useful if you only need to regenerate interface configs, for example.</t>
+          <t>Toggle which config sections to generate (Yes/No). The top-level 'base_config' flag controls whether the base config runs at all. Sub-features (aaa, snmp, ntp, dhcp_snooping, spanning_tree, banner) let you skip individual sections within the base config — useful if those sections are already deployed or managed by another system.</t>
         </is>
       </c>
     </row>
@@ -3080,7 +3080,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3118,14 +3118,14 @@
       </c>
       <c r="C2" s="12" t="inlineStr">
         <is>
-          <t>Base switch config — hostname, AAA, NTP, SNMP, STP, SSH hardening</t>
+          <t>Base switch config — hostname, SSH hardening, management interface, IP routing off</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>vlans</t>
+          <t>aaa</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
@@ -3135,14 +3135,14 @@
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>VLAN definitions</t>
+          <t>AAA — aaa new-model, TACACS+ group, authentication and authorisation commands</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
-          <t>interfaces</t>
+          <t>snmp</t>
         </is>
       </c>
       <c r="B4" s="12" t="inlineStr">
@@ -3152,22 +3152,124 @@
       </c>
       <c r="C4" s="12" t="inlineStr">
         <is>
-          <t>Interface config — access, trunk, and unused ports</t>
+          <t>SNMPv3 — groups, users, host, location and contact (requires SNMPv3 credentials in Global Settings)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
+          <t>ntp</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>NTP server configuration (requires NTP servers in Global Settings)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>dhcp_snooping</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>DHCP snooping — enabled globally across all VLANs</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>spanning_tree</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Spanning tree — mode rapid-pvst, extend system-id, portfast BPDUguard default</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>banner</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Banner MOTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>vlans</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>VLAN definitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>interfaces</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Interface config — access, trunk, and unused ports</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
           <t>acls</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C11" s="13" t="inlineStr">
         <is>
           <t>IP access control lists — VTY and SNMP access restriction</t>
         </is>

</xml_diff>